<commit_message>
Completely clean up hallucination terminology and replace with non-overlapping spurious FPs across error breakdown and revision plan
</commit_message>
<xml_diff>
--- a/publication/results/error_analysis/error_breakdown_summary.xlsx
+++ b/publication/results/error_analysis/error_breakdown_summary.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_Sonnet_FAERS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_LLaMA4_FAERS" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_LLaMA4_VAERS" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hallucination_Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spurious_Non_Overlap_Summary" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total_Hallucinations</t>
+          <t>Total_Spurious_Non_Overlap</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Top_Hallucinated_Terms</t>
+          <t>Top_Spurious_Terms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: Update evaluation scripts and generate supplementary materials
- Implemented Two-Tier Evaluation Framework (Strict vs ADE-Eval)
- Updated BioBERT results to report mean/std across 10-fold CV, 4-fold LOO, and 5 random seeds (Seed 42 default)
- Updated evaluate_three_schemes.py and analyze_error_breakdown.py scripts
- Re-generated three_schemes_summary.xlsx and error_breakdown_summary.xlsx
- Drafted supplementary_materials.md with annotation guidelines and BioBERT rationale
- Updated manuscript_revision_plan.md with the latest metric breakdown
</commit_message>
<xml_diff>
--- a/publication/results/error_analysis/error_breakdown_summary.xlsx
+++ b/publication/results/error_analysis/error_breakdown_summary.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category_C_Granularity" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_Sonnet_FAERS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_LLaMA4_FAERS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_LLaMA4_VAERS" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spurious_Non_Overlap_Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_LLaMA4_JSON_FAERS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion_LLaMA4_VAERS" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spurious_Non_Overlap_Summary" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1320,7 +1321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1438,7 +1439,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BioBERT (Fold 0)</t>
+          <t>BioBERT (Seed 42, Fold 0)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1447,37 +1448,37 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>383</v>
+        <v>157</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5223</v>
+        <v>0.5232</v>
       </c>
       <c r="E3" t="n">
-        <v>0.5185</v>
+        <v>0.5294</v>
       </c>
       <c r="F3" t="n">
-        <v>9.4</v>
+        <v>7.01</v>
       </c>
       <c r="G3" t="n">
-        <v>46.48</v>
+        <v>52.23</v>
       </c>
       <c r="H3" t="n">
-        <v>44.13</v>
+        <v>40.76</v>
       </c>
       <c r="I3" t="n">
-        <v>1.31</v>
+        <v>1.27</v>
       </c>
       <c r="J3" t="n">
-        <v>0.52</v>
+        <v>3.82</v>
       </c>
       <c r="K3" t="n">
-        <v>3.92</v>
+        <v>3.18</v>
       </c>
       <c r="L3" t="n">
-        <v>92.95</v>
+        <v>91.72</v>
       </c>
       <c r="M3" t="n">
-        <v>1.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1528,7 +1529,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LLaMA 4</t>
+          <t>LLaMA 4 (JSON)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1537,81 +1538,126 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5420</v>
+        <v>4511</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4713</v>
+        <v>0.4654</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4667</v>
+        <v>0.451</v>
       </c>
       <c r="F5" t="n">
-        <v>7.84</v>
+        <v>8.25</v>
       </c>
       <c r="G5" t="n">
-        <v>37.55</v>
+        <v>34.74</v>
       </c>
       <c r="H5" t="n">
-        <v>54.61</v>
+        <v>57.02</v>
       </c>
       <c r="I5" t="n">
-        <v>0.61</v>
+        <v>0.51</v>
       </c>
       <c r="J5" t="n">
-        <v>1.37</v>
+        <v>0.75</v>
       </c>
       <c r="K5" t="n">
-        <v>6.59</v>
+        <v>3.19</v>
       </c>
       <c r="L5" t="n">
-        <v>85.52</v>
+        <v>90.42</v>
       </c>
       <c r="M5" t="n">
-        <v>5.92</v>
+        <v>5.12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LLaMA 4</t>
+          <t>LLaMA 4 (Tagged)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>FAERS</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5420</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.4713</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.4667</v>
+      </c>
+      <c r="F6" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="G6" t="n">
+        <v>37.55</v>
+      </c>
+      <c r="H6" t="n">
+        <v>54.61</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="K6" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="L6" t="n">
+        <v>85.52</v>
+      </c>
+      <c r="M6" t="n">
+        <v>5.92</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LLaMA 4 (Tagged)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>VAERS</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C7" t="n">
         <v>7608</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>0.4197</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E7" t="n">
         <v>0.4</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F7" t="n">
         <v>5.48</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G7" t="n">
         <v>30.98</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H7" t="n">
         <v>63.54</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I7" t="n">
         <v>0.79</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J7" t="n">
         <v>0.05</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K7" t="n">
         <v>6.23</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L7" t="n">
         <v>89.56</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M7" t="n">
         <v>3.36</v>
       </c>
     </row>
@@ -2856,7 +2902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2872,30 +2918,60 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>COD</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>DOSE</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>DRUG</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>DX</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>HX</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>INDICATION</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>LAB</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>VAX</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>All</t>
         </is>
@@ -2908,193 +2984,595 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6809</v>
+        <v>826</v>
       </c>
       <c r="C2" t="n">
-        <v>669</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>919</v>
+        <v>128</v>
       </c>
       <c r="E2" t="n">
-        <v>1050</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="G2" t="n">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="H2" t="n">
-        <v>9615</v>
+        <v>120</v>
+      </c>
+      <c r="I2" t="n">
+        <v>78</v>
+      </c>
+      <c r="J2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K2" t="n">
+        <v>24</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M2" t="n">
+        <v>186</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1571</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>HX</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
         <v>10</v>
-      </c>
-      <c r="D3" t="n">
-        <v>9</v>
-      </c>
-      <c r="E3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>6</v>
-      </c>
-      <c r="H3" t="n">
-        <v>153</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>LAB</t>
+          <t>COD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>182</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>898</v>
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>STATUS</t>
+          <t>DOSE</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>234</v>
       </c>
       <c r="F5" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H5" t="n">
-        <v>109</v>
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>7</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>256</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>DRUG</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C6" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>105</v>
       </c>
       <c r="F6" t="n">
+        <v>710</v>
+      </c>
+      <c r="G6" t="n">
+        <v>482</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
         <v>5</v>
       </c>
-      <c r="G6" t="n">
-        <v>63</v>
-      </c>
-      <c r="H6" t="n">
-        <v>130</v>
+      <c r="N6" t="n">
+        <v>1324</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>VAX</t>
+          <t>DX</t>
         </is>
       </c>
       <c r="B7" t="n">
+        <v>36</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>167</v>
+      </c>
+      <c r="F7" t="n">
+        <v>442</v>
+      </c>
+      <c r="G7" t="n">
+        <v>36</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" t="n">
+        <v>8</v>
+      </c>
+      <c r="J7" t="n">
+        <v>38</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
         <v>29</v>
       </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>9</v>
-      </c>
-      <c r="F7" t="n">
-        <v>34</v>
-      </c>
-      <c r="G7" t="n">
-        <v>16</v>
-      </c>
-      <c r="H7" t="n">
-        <v>94</v>
+      <c r="N7" t="n">
+        <v>770</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
+          <t>HX</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>126</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>11</v>
+      </c>
+      <c r="F8" t="n">
+        <v>106</v>
+      </c>
+      <c r="G8" t="n">
+        <v>36</v>
+      </c>
+      <c r="H8" t="n">
+        <v>75</v>
+      </c>
+      <c r="I8" t="n">
+        <v>205</v>
+      </c>
+      <c r="J8" t="n">
+        <v>25</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>8</v>
+      </c>
+      <c r="N8" t="n">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>INDICATION</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>11</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>24</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>LAB</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>485</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>775</v>
+      </c>
+      <c r="F10" t="n">
+        <v>58</v>
+      </c>
+      <c r="G10" t="n">
+        <v>253</v>
+      </c>
+      <c r="H10" t="n">
+        <v>15</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>658</v>
+      </c>
+      <c r="K10" t="n">
+        <v>10</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" t="n">
+        <v>101</v>
+      </c>
+      <c r="N10" t="n">
+        <v>2360</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>45</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>14</v>
+      </c>
+      <c r="N13" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
           <t>All</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>7102</v>
-      </c>
-      <c r="C8" t="n">
-        <v>739</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1129</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1099</v>
-      </c>
-      <c r="F8" t="n">
-        <v>771</v>
-      </c>
-      <c r="G8" t="n">
-        <v>159</v>
-      </c>
-      <c r="H8" t="n">
-        <v>10999</v>
+      <c r="B14" t="n">
+        <v>1539</v>
+      </c>
+      <c r="C14" t="n">
+        <v>16</v>
+      </c>
+      <c r="D14" t="n">
+        <v>137</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1305</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1389</v>
+      </c>
+      <c r="G14" t="n">
+        <v>841</v>
+      </c>
+      <c r="H14" t="n">
+        <v>249</v>
+      </c>
+      <c r="I14" t="n">
+        <v>301</v>
+      </c>
+      <c r="J14" t="n">
+        <v>835</v>
+      </c>
+      <c r="K14" t="n">
+        <v>37</v>
+      </c>
+      <c r="L14" t="n">
+        <v>14</v>
+      </c>
+      <c r="M14" t="n">
+        <v>349</v>
+      </c>
+      <c r="N14" t="n">
+        <v>7012</v>
       </c>
     </row>
   </sheetData>
@@ -3108,12 +3586,264 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Gold_Category</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>HX</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>LAB</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>VAX</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6809</v>
+      </c>
+      <c r="C2" t="n">
+        <v>669</v>
+      </c>
+      <c r="D2" t="n">
+        <v>919</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F2" t="n">
+        <v>104</v>
+      </c>
+      <c r="G2" t="n">
+        <v>64</v>
+      </c>
+      <c r="H2" t="n">
+        <v>9615</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>HX</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>114</v>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>LAB</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>55</v>
+      </c>
+      <c r="C4" t="n">
+        <v>27</v>
+      </c>
+      <c r="D4" t="n">
+        <v>182</v>
+      </c>
+      <c r="E4" t="n">
+        <v>24</v>
+      </c>
+      <c r="F4" t="n">
+        <v>600</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" t="n">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>82</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>19</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C6" t="n">
+        <v>32</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>63</v>
+      </c>
+      <c r="H6" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>VAX</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>29</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" t="n">
+        <v>34</v>
+      </c>
+      <c r="G7" t="n">
+        <v>16</v>
+      </c>
+      <c r="H7" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7102</v>
+      </c>
+      <c r="C8" t="n">
+        <v>739</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1129</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1099</v>
+      </c>
+      <c r="F8" t="n">
+        <v>771</v>
+      </c>
+      <c r="G8" t="n">
+        <v>159</v>
+      </c>
+      <c r="H8" t="n">
+        <v>10999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>Model</t>
         </is>
       </c>
@@ -3166,7 +3896,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BioBERT (Fold 0)</t>
+          <t>BioBERT (Seed 42, Fold 0)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3175,16 +3905,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>556</v>
+        <v>203</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{'AE': 284, 'LAB': 95, 'STATUS': 83, 'VAX': 72, 'TX': 20}</t>
+          <t>{'AE': 85, 'LAB': 58, 'STATUS': 24, 'TX': 18, 'VAX': 16}</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{'hospitalization': 17, 'ROTATEQ': 8, 'death': 7, 'serious': 6, 'ice': 5, 'medically significant': 4, 'stable condition': 4, 'vomiting': 3, 'discharge': 3, 'pregnancy': 3}</t>
+          <t>{'death': 5, 'herpes zoster vaccine': 3, 'GARDASIL': 3, 'sleeping': 2, 'ENBREL': 2, 'near death': 2, 'very upset': 2, 'no reported medical history': 2, 'abscess': 2, 'SpO2': 2}</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3946,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LLaMA 4</t>
+          <t>LLaMA 4 (JSON)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3225,39 +3955,64 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15269</v>
+        <v>8166</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>{'AE': 5729, 'DRUG': 4165, 'HX': 1323, 'INDICATION': 1056, 'DX': 986}</t>
+          <t>{'AE': 1699, 'DRUG': 1362, 'DX': 1064, 'STATUS': 1026, 'HX': 976}</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{'Aimovig': 682, 'Vidaza': 339, 'tramadol': 217, 'Azacitidine': 211, 'cerebrovascular accident': 204, 'baricitinib': 136, 'unknown': 128, 'migraine': 127, 'hypoglycemia': 127, 'hypoglycaemia': 125}</t>
+          <t>{'Aimovig': 259, 'unknown': 179, 'Vidaza': 139, 'unknown indication': 109, 'tramadol': 97, 'migraine': 80, 'rheumatoid arthritis': 68, 'cardiac arrest': 63, 'Azacitidine': 63, 'baricitinib': 59}</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LLaMA 4</t>
+          <t>LLaMA 4 (Tagged)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>FAERS</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>15269</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{'AE': 5729, 'DRUG': 4165, 'HX': 1323, 'INDICATION': 1056, 'DX': 986}</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{'Aimovig': 682, 'Vidaza': 339, 'tramadol': 217, 'Azacitidine': 211, 'cerebrovascular accident': 204, 'baricitinib': 136, 'unknown': 128, 'migraine': 127, 'hypoglycemia': 127, 'hypoglycaemia': 125}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LLaMA 4 (Tagged)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>VAERS</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C7" t="n">
         <v>5666</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>{'LAB': 2062, 'TX': 1100, 'AE': 1088, 'VAX': 700, 'STATUS': 542}</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>{'symptoms': 153, 'vaccine': 126, 'vaccination': 80, 'treatment': 61, 'medical history': 37, 'GlaxoSmithKline': 33, 'hospitalization': 32, 'MMRV': 32, 'emergency room': 27, 'MMR + V': 26}</t>
         </is>

</xml_diff>